<commit_message>
Actualizar Wage11_PROCESADO.xlsx con datos del analisis final
</commit_message>
<xml_diff>
--- a/Wage11_PROCESADO.xlsx
+++ b/Wage11_PROCESADO.xlsx
@@ -711,7 +711,9 @@
       <c r="D5" t="n">
         <v>45</v>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F5" t="n">
         <v>43</v>
       </c>
@@ -1750,7 +1752,9 @@
       <c r="F22" t="n">
         <v>40</v>
       </c>
-      <c r="G22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>12</v>
+      </c>
       <c r="H22" t="n">
         <v>18</v>
       </c>
@@ -1784,7 +1788,9 @@
       <c r="R22" t="n">
         <v>15.6</v>
       </c>
-      <c r="S22" t="inlineStr"/>
+      <c r="S22" t="n">
+        <v>0.631578947368421</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1912,7 +1918,9 @@
       <c r="A25" t="n">
         <v>25</v>
       </c>
-      <c r="B25" t="inlineStr"/>
+      <c r="B25" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C25" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -1954,11 +1962,15 @@
       <c r="O25" t="n">
         <v>0</v>
       </c>
-      <c r="P25" t="inlineStr"/>
+      <c r="P25" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q25" t="n">
         <v>0.1716486370112518</v>
       </c>
-      <c r="R25" t="inlineStr"/>
+      <c r="R25" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S25" t="n">
         <v>1.333333333333333</v>
       </c>
@@ -2008,7 +2020,9 @@
       <c r="N26" t="n">
         <v>1</v>
       </c>
-      <c r="O26" t="inlineStr"/>
+      <c r="O26" t="n">
+        <v>2</v>
+      </c>
       <c r="P26" t="n">
         <v>0.3391096504332238</v>
       </c>
@@ -2241,7 +2255,9 @@
       <c r="K30" t="n">
         <v>1</v>
       </c>
-      <c r="L30" t="inlineStr"/>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
       <c r="M30" t="n">
         <v>1</v>
       </c>
@@ -2725,7 +2741,9 @@
       <c r="K38" t="n">
         <v>1</v>
       </c>
-      <c r="L38" t="inlineStr"/>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
       <c r="M38" t="n">
         <v>0</v>
       </c>
@@ -2952,7 +2970,9 @@
       <c r="F42" t="n">
         <v>40</v>
       </c>
-      <c r="G42" t="inlineStr"/>
+      <c r="G42" t="n">
+        <v>12</v>
+      </c>
       <c r="H42" t="n">
         <v>18</v>
       </c>
@@ -2986,7 +3006,9 @@
       <c r="R42" t="n">
         <v>20.2</v>
       </c>
-      <c r="S42" t="inlineStr"/>
+      <c r="S42" t="n">
+        <v>0.631578947368421</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3073,7 +3095,9 @@
       <c r="G44" t="n">
         <v>18</v>
       </c>
-      <c r="H44" t="inlineStr"/>
+      <c r="H44" t="n">
+        <v>11</v>
+      </c>
       <c r="I44" t="n">
         <v>1</v>
       </c>
@@ -3104,7 +3128,9 @@
       <c r="R44" t="n">
         <v>9.781818181818181</v>
       </c>
-      <c r="S44" t="inlineStr"/>
+      <c r="S44" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3310,7 +3336,9 @@
       <c r="F48" t="n">
         <v>22</v>
       </c>
-      <c r="G48" t="inlineStr"/>
+      <c r="G48" t="n">
+        <v>12</v>
+      </c>
       <c r="H48" t="n">
         <v>11</v>
       </c>
@@ -3344,7 +3372,9 @@
       <c r="R48" t="n">
         <v>18.025</v>
       </c>
-      <c r="S48" t="inlineStr"/>
+      <c r="S48" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3611,7 +3641,9 @@
       <c r="F53" t="n">
         <v>40</v>
       </c>
-      <c r="G53" t="inlineStr"/>
+      <c r="G53" t="n">
+        <v>12</v>
+      </c>
       <c r="H53" t="n">
         <v>9</v>
       </c>
@@ -3645,7 +3677,9 @@
       <c r="R53" t="n">
         <v>17.5</v>
       </c>
-      <c r="S53" t="inlineStr"/>
+      <c r="S53" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -3805,7 +3839,9 @@
       <c r="K56" t="n">
         <v>1</v>
       </c>
-      <c r="L56" t="inlineStr"/>
+      <c r="L56" t="n">
+        <v>0</v>
+      </c>
       <c r="M56" t="n">
         <v>0</v>
       </c>
@@ -4422,7 +4458,9 @@
       <c r="N66" t="n">
         <v>0</v>
       </c>
-      <c r="O66" t="inlineStr"/>
+      <c r="O66" t="n">
+        <v>2</v>
+      </c>
       <c r="P66" t="n">
         <v>0.2420077681505826</v>
       </c>
@@ -4542,7 +4580,9 @@
       <c r="N68" t="n">
         <v>1</v>
       </c>
-      <c r="O68" t="inlineStr"/>
+      <c r="O68" t="n">
+        <v>2</v>
+      </c>
       <c r="P68" t="n">
         <v>0.235733492680012</v>
       </c>
@@ -4601,7 +4641,9 @@
       <c r="N69" t="n">
         <v>1</v>
       </c>
-      <c r="O69" t="inlineStr"/>
+      <c r="O69" t="n">
+        <v>2</v>
+      </c>
       <c r="P69" t="n">
         <v>0.1673140125485509</v>
       </c>
@@ -4691,7 +4733,9 @@
       <c r="D71" t="n">
         <v>50</v>
       </c>
-      <c r="E71" t="inlineStr"/>
+      <c r="E71" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F71" t="n">
         <v>41</v>
       </c>
@@ -4954,7 +4998,9 @@
       <c r="K75" t="n">
         <v>1</v>
       </c>
-      <c r="L75" t="inlineStr"/>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
       <c r="M75" t="n">
         <v>1</v>
       </c>
@@ -5120,7 +5166,9 @@
       <c r="F78" t="n">
         <v>30</v>
       </c>
-      <c r="G78" t="inlineStr"/>
+      <c r="G78" t="n">
+        <v>12</v>
+      </c>
       <c r="H78" t="n">
         <v>9</v>
       </c>
@@ -5154,7 +5202,9 @@
       <c r="R78" t="n">
         <v>56.46666666666667</v>
       </c>
-      <c r="S78" t="inlineStr"/>
+      <c r="S78" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -5709,7 +5759,9 @@
       <c r="A88" t="n">
         <v>95</v>
       </c>
-      <c r="B88" t="inlineStr"/>
+      <c r="B88" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C88" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -5751,11 +5803,15 @@
       <c r="O88" t="n">
         <v>8</v>
       </c>
-      <c r="P88" t="inlineStr"/>
+      <c r="P88" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q88" t="n">
         <v>1.481598761570805</v>
       </c>
-      <c r="R88" t="inlineStr"/>
+      <c r="R88" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S88" t="n">
         <v>0.7058823529411765</v>
       </c>
@@ -6451,7 +6507,9 @@
       <c r="G100" t="n">
         <v>14</v>
       </c>
-      <c r="H100" t="inlineStr"/>
+      <c r="H100" t="n">
+        <v>11</v>
+      </c>
       <c r="I100" t="n">
         <v>1</v>
       </c>
@@ -6482,7 +6540,9 @@
       <c r="R100" t="n">
         <v>27.775</v>
       </c>
-      <c r="S100" t="inlineStr"/>
+      <c r="S100" t="n">
+        <v>1.166666666666667</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -6625,7 +6685,9 @@
       <c r="F103" t="n">
         <v>22</v>
       </c>
-      <c r="G103" t="inlineStr"/>
+      <c r="G103" t="n">
+        <v>12</v>
+      </c>
       <c r="H103" t="n">
         <v>11</v>
       </c>
@@ -6659,7 +6721,9 @@
       <c r="R103" t="n">
         <v>13.825</v>
       </c>
-      <c r="S103" t="inlineStr"/>
+      <c r="S103" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -6682,7 +6746,9 @@
       <c r="F104" t="n">
         <v>38</v>
       </c>
-      <c r="G104" t="inlineStr"/>
+      <c r="G104" t="n">
+        <v>12</v>
+      </c>
       <c r="H104" t="n">
         <v>15</v>
       </c>
@@ -6716,7 +6782,9 @@
       <c r="R104" t="n">
         <v>35.94736842105263</v>
       </c>
-      <c r="S104" t="inlineStr"/>
+      <c r="S104" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -6739,7 +6807,9 @@
       <c r="F105" t="n">
         <v>40</v>
       </c>
-      <c r="G105" t="inlineStr"/>
+      <c r="G105" t="n">
+        <v>12</v>
+      </c>
       <c r="H105" t="n">
         <v>10</v>
       </c>
@@ -6773,13 +6843,17 @@
       <c r="R105" t="n">
         <v>35.6</v>
       </c>
-      <c r="S105" t="inlineStr"/>
+      <c r="S105" t="n">
+        <v>1.090909090909091</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
         <v>116</v>
       </c>
-      <c r="B106" t="inlineStr"/>
+      <c r="B106" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C106" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -6821,11 +6895,15 @@
       <c r="O106" t="n">
         <v>7</v>
       </c>
-      <c r="P106" t="inlineStr"/>
+      <c r="P106" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q106" t="n">
         <v>0.04065362455529643</v>
       </c>
-      <c r="R106" t="inlineStr"/>
+      <c r="R106" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S106" t="n">
         <v>7</v>
       </c>
@@ -7049,7 +7127,9 @@
       <c r="K110" t="n">
         <v>1</v>
       </c>
-      <c r="L110" t="inlineStr"/>
+      <c r="L110" t="n">
+        <v>0</v>
+      </c>
       <c r="M110" t="n">
         <v>0</v>
       </c>
@@ -7259,7 +7339,9 @@
       <c r="A114" t="n">
         <v>124</v>
       </c>
-      <c r="B114" t="inlineStr"/>
+      <c r="B114" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C114" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -7301,11 +7383,15 @@
       <c r="O114" t="n">
         <v>2</v>
       </c>
-      <c r="P114" t="inlineStr"/>
+      <c r="P114" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q114" t="n">
         <v>-2.055266574739989</v>
       </c>
-      <c r="R114" t="inlineStr"/>
+      <c r="R114" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S114" t="n">
         <v>1.1</v>
       </c>
@@ -7375,7 +7461,9 @@
       <c r="A116" t="n">
         <v>126</v>
       </c>
-      <c r="B116" t="inlineStr"/>
+      <c r="B116" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C116" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -7417,11 +7505,15 @@
       <c r="O116" t="n">
         <v>3</v>
       </c>
-      <c r="P116" t="inlineStr"/>
+      <c r="P116" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q116" t="n">
         <v>-1.662281537372123</v>
       </c>
-      <c r="R116" t="inlineStr"/>
+      <c r="R116" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S116" t="n">
         <v>0.7333333333333333</v>
       </c>
@@ -7508,7 +7600,9 @@
       <c r="F118" t="n">
         <v>37</v>
       </c>
-      <c r="G118" t="inlineStr"/>
+      <c r="G118" t="n">
+        <v>12</v>
+      </c>
       <c r="H118" t="n">
         <v>17</v>
       </c>
@@ -7542,7 +7636,9 @@
       <c r="R118" t="n">
         <v>19.16</v>
       </c>
-      <c r="S118" t="inlineStr"/>
+      <c r="S118" t="n">
+        <v>0.6666666666666666</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -7565,7 +7661,9 @@
       <c r="F119" t="n">
         <v>42</v>
       </c>
-      <c r="G119" t="inlineStr"/>
+      <c r="G119" t="n">
+        <v>12</v>
+      </c>
       <c r="H119" t="n">
         <v>8</v>
       </c>
@@ -7599,7 +7697,9 @@
       <c r="R119" t="n">
         <v>27.68</v>
       </c>
-      <c r="S119" t="inlineStr"/>
+      <c r="S119" t="n">
+        <v>1.333333333333333</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -7849,7 +7949,9 @@
       <c r="A124" t="n">
         <v>134</v>
       </c>
-      <c r="B124" t="inlineStr"/>
+      <c r="B124" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C124" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -7891,11 +7993,15 @@
       <c r="O124" t="n">
         <v>1</v>
       </c>
-      <c r="P124" t="inlineStr"/>
+      <c r="P124" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q124" t="n">
         <v>-0.6143214377244803</v>
       </c>
-      <c r="R124" t="inlineStr"/>
+      <c r="R124" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S124" t="n">
         <v>0.8666666666666667</v>
       </c>
@@ -7921,7 +8027,9 @@
       <c r="F125" t="n">
         <v>24</v>
       </c>
-      <c r="G125" t="inlineStr"/>
+      <c r="G125" t="n">
+        <v>12</v>
+      </c>
       <c r="H125" t="n">
         <v>3</v>
       </c>
@@ -7955,7 +8063,9 @@
       <c r="R125" t="n">
         <v>34.375</v>
       </c>
-      <c r="S125" t="inlineStr"/>
+      <c r="S125" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -8401,7 +8511,9 @@
       <c r="F133" t="n">
         <v>30</v>
       </c>
-      <c r="G133" t="inlineStr"/>
+      <c r="G133" t="n">
+        <v>12</v>
+      </c>
       <c r="H133" t="n">
         <v>8</v>
       </c>
@@ -8435,7 +8547,9 @@
       <c r="R133" t="n">
         <v>11.4</v>
       </c>
-      <c r="S133" t="inlineStr"/>
+      <c r="S133" t="n">
+        <v>1.333333333333333</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -8522,7 +8636,9 @@
       <c r="G135" t="n">
         <v>12</v>
       </c>
-      <c r="H135" t="inlineStr"/>
+      <c r="H135" t="n">
+        <v>11</v>
+      </c>
       <c r="I135" t="n">
         <v>1</v>
       </c>
@@ -8553,7 +8669,9 @@
       <c r="R135" t="n">
         <v>31.25</v>
       </c>
-      <c r="S135" t="inlineStr"/>
+      <c r="S135" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -9128,7 +9246,9 @@
       <c r="G145" t="n">
         <v>12</v>
       </c>
-      <c r="H145" t="inlineStr"/>
+      <c r="H145" t="n">
+        <v>11</v>
+      </c>
       <c r="I145" t="n">
         <v>7</v>
       </c>
@@ -9159,7 +9279,9 @@
       <c r="R145" t="n">
         <v>16.25</v>
       </c>
-      <c r="S145" t="inlineStr"/>
+      <c r="S145" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -9185,7 +9307,9 @@
       <c r="G146" t="n">
         <v>18</v>
       </c>
-      <c r="H146" t="inlineStr"/>
+      <c r="H146" t="n">
+        <v>11</v>
+      </c>
       <c r="I146" t="n">
         <v>14</v>
       </c>
@@ -9216,7 +9340,9 @@
       <c r="R146" t="n">
         <v>47.475</v>
       </c>
-      <c r="S146" t="inlineStr"/>
+      <c r="S146" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -9780,7 +9906,9 @@
       <c r="D156" t="n">
         <v>40</v>
       </c>
-      <c r="E156" t="inlineStr"/>
+      <c r="E156" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F156" t="n">
         <v>31</v>
       </c>
@@ -10477,7 +10605,9 @@
       <c r="N167" t="n">
         <v>0</v>
       </c>
-      <c r="O167" t="inlineStr"/>
+      <c r="O167" t="n">
+        <v>2</v>
+      </c>
       <c r="P167" t="n">
         <v>0.09501045712578426</v>
       </c>
@@ -10769,7 +10899,9 @@
       <c r="K172" t="n">
         <v>1</v>
       </c>
-      <c r="L172" t="inlineStr"/>
+      <c r="L172" t="n">
+        <v>0</v>
+      </c>
       <c r="M172" t="n">
         <v>1</v>
       </c>
@@ -11182,7 +11314,9 @@
       <c r="G179" t="n">
         <v>18</v>
       </c>
-      <c r="H179" t="inlineStr"/>
+      <c r="H179" t="n">
+        <v>11</v>
+      </c>
       <c r="I179" t="n">
         <v>8</v>
       </c>
@@ -11213,7 +11347,9 @@
       <c r="R179" t="n">
         <v>28.6</v>
       </c>
-      <c r="S179" t="inlineStr"/>
+      <c r="S179" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" t="n">
@@ -11300,7 +11436,9 @@
       <c r="G181" t="n">
         <v>12</v>
       </c>
-      <c r="H181" t="inlineStr"/>
+      <c r="H181" t="n">
+        <v>11</v>
+      </c>
       <c r="I181" t="n">
         <v>18</v>
       </c>
@@ -11331,7 +11469,9 @@
       <c r="R181" t="n">
         <v>17</v>
       </c>
-      <c r="S181" t="inlineStr"/>
+      <c r="S181" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="n">
@@ -11735,7 +11875,9 @@
       <c r="K188" t="n">
         <v>1</v>
       </c>
-      <c r="L188" t="inlineStr"/>
+      <c r="L188" t="n">
+        <v>0</v>
+      </c>
       <c r="M188" t="n">
         <v>0</v>
       </c>
@@ -12065,7 +12207,9 @@
       <c r="A194" t="n">
         <v>209</v>
       </c>
-      <c r="B194" t="inlineStr"/>
+      <c r="B194" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C194" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -12107,11 +12251,15 @@
       <c r="O194" t="n">
         <v>1</v>
       </c>
-      <c r="P194" t="inlineStr"/>
+      <c r="P194" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q194" t="n">
         <v>0.5646336743791178</v>
       </c>
-      <c r="R194" t="inlineStr"/>
+      <c r="R194" t="n">
+        <v>16.53636363636364</v>
+      </c>
       <c r="S194" t="n">
         <v>1.363636363636364</v>
       </c>
@@ -12274,7 +12422,9 @@
       <c r="K197" t="n">
         <v>1</v>
       </c>
-      <c r="L197" t="inlineStr"/>
+      <c r="L197" t="n">
+        <v>0</v>
+      </c>
       <c r="M197" t="n">
         <v>1</v>
       </c>
@@ -12333,7 +12483,9 @@
       <c r="K198" t="n">
         <v>1</v>
       </c>
-      <c r="L198" t="inlineStr"/>
+      <c r="L198" t="n">
+        <v>0</v>
+      </c>
       <c r="M198" t="n">
         <v>0</v>
       </c>
@@ -12438,7 +12590,9 @@
       <c r="F200" t="n">
         <v>28</v>
       </c>
-      <c r="G200" t="inlineStr"/>
+      <c r="G200" t="n">
+        <v>12</v>
+      </c>
       <c r="H200" t="n">
         <v>7</v>
       </c>
@@ -12472,7 +12626,9 @@
       <c r="R200" t="n">
         <v>8.625</v>
       </c>
-      <c r="S200" t="inlineStr"/>
+      <c r="S200" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="n">
@@ -12495,7 +12651,9 @@
       <c r="F201" t="n">
         <v>38</v>
       </c>
-      <c r="G201" t="inlineStr"/>
+      <c r="G201" t="n">
+        <v>12</v>
+      </c>
       <c r="H201" t="n">
         <v>1</v>
       </c>
@@ -12529,13 +12687,17 @@
       <c r="R201" t="n">
         <v>12.7</v>
       </c>
-      <c r="S201" t="inlineStr"/>
+      <c r="S201" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="n">
         <v>220</v>
       </c>
-      <c r="B202" t="inlineStr"/>
+      <c r="B202" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C202" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -12577,11 +12739,15 @@
       <c r="O202" t="n">
         <v>5</v>
       </c>
-      <c r="P202" t="inlineStr"/>
+      <c r="P202" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q202" t="n">
         <v>-1.662281537372123</v>
       </c>
-      <c r="R202" t="inlineStr"/>
+      <c r="R202" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S202" t="n">
         <v>1</v>
       </c>
@@ -12956,7 +13122,9 @@
       <c r="A209" t="n">
         <v>227</v>
       </c>
-      <c r="B209" t="inlineStr"/>
+      <c r="B209" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C209" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -12998,11 +13166,15 @@
       <c r="O209" t="n">
         <v>1</v>
       </c>
-      <c r="P209" t="inlineStr"/>
+      <c r="P209" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q209" t="n">
         <v>0.4336386619231625</v>
       </c>
-      <c r="R209" t="inlineStr"/>
+      <c r="R209" t="n">
+        <v>15.15833333333333</v>
+      </c>
       <c r="S209" t="n">
         <v>1.6</v>
       </c>
@@ -13470,7 +13642,9 @@
       <c r="K217" t="n">
         <v>1</v>
       </c>
-      <c r="L217" t="inlineStr"/>
+      <c r="L217" t="n">
+        <v>0</v>
+      </c>
       <c r="M217" t="n">
         <v>0</v>
       </c>
@@ -13636,7 +13810,9 @@
       <c r="F220" t="n">
         <v>46</v>
       </c>
-      <c r="G220" t="inlineStr"/>
+      <c r="G220" t="n">
+        <v>12</v>
+      </c>
       <c r="H220" t="n">
         <v>6</v>
       </c>
@@ -13670,13 +13846,17 @@
       <c r="R220" t="n">
         <v>12.71428571428571</v>
       </c>
-      <c r="S220" t="inlineStr"/>
+      <c r="S220" t="n">
+        <v>1.714285714285714</v>
+      </c>
     </row>
     <row r="221">
       <c r="A221" t="n">
         <v>240</v>
       </c>
-      <c r="B221" t="inlineStr"/>
+      <c r="B221" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C221" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -13718,11 +13898,15 @@
       <c r="O221" t="n">
         <v>1</v>
       </c>
-      <c r="P221" t="inlineStr"/>
+      <c r="P221" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q221" t="n">
         <v>0.8266236992910285</v>
       </c>
-      <c r="R221" t="inlineStr"/>
+      <c r="R221" t="n">
+        <v>16.24107142857143</v>
+      </c>
       <c r="S221" t="n">
         <v>0.6666666666666666</v>
       </c>
@@ -14443,7 +14627,9 @@
       <c r="N233" t="n">
         <v>1</v>
       </c>
-      <c r="O233" t="inlineStr"/>
+      <c r="O233" t="n">
+        <v>2</v>
+      </c>
       <c r="P233" t="n">
         <v>0.2942933970720048</v>
       </c>
@@ -14583,7 +14769,9 @@
       <c r="A236" t="n">
         <v>257</v>
       </c>
-      <c r="B236" t="inlineStr"/>
+      <c r="B236" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C236" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -14625,11 +14813,15 @@
       <c r="O236" t="n">
         <v>8</v>
       </c>
-      <c r="P236" t="inlineStr"/>
+      <c r="P236" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q236" t="n">
         <v>-2.3172565996519</v>
       </c>
-      <c r="R236" t="inlineStr"/>
+      <c r="R236" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S236" t="n">
         <v>0.6666666666666666</v>
       </c>
@@ -14638,7 +14830,9 @@
       <c r="A237" t="n">
         <v>258</v>
       </c>
-      <c r="B237" t="inlineStr"/>
+      <c r="B237" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C237" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -14680,11 +14874,15 @@
       <c r="O237" t="n">
         <v>2</v>
       </c>
-      <c r="P237" t="inlineStr"/>
+      <c r="P237" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q237" t="n">
         <v>0.3026436494672071</v>
       </c>
-      <c r="R237" t="inlineStr"/>
+      <c r="R237" t="n">
+        <v>21.65476190476191</v>
+      </c>
       <c r="S237" t="n">
         <v>2.125</v>
       </c>
@@ -15423,7 +15621,9 @@
       <c r="A250" t="n">
         <v>271</v>
       </c>
-      <c r="B250" t="inlineStr"/>
+      <c r="B250" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C250" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -15465,11 +15665,15 @@
       <c r="O250" t="n">
         <v>2</v>
       </c>
-      <c r="P250" t="inlineStr"/>
+      <c r="P250" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q250" t="n">
         <v>-1.924271562284034</v>
       </c>
-      <c r="R250" t="inlineStr"/>
+      <c r="R250" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S250" t="n">
         <v>2</v>
       </c>
@@ -15678,7 +15882,9 @@
       <c r="F254" t="n">
         <v>39</v>
       </c>
-      <c r="G254" t="inlineStr"/>
+      <c r="G254" t="n">
+        <v>12</v>
+      </c>
       <c r="H254" t="n">
         <v>14</v>
       </c>
@@ -15712,7 +15918,9 @@
       <c r="R254" t="n">
         <v>33.65</v>
       </c>
-      <c r="S254" t="inlineStr"/>
+      <c r="S254" t="n">
+        <v>0.8</v>
+      </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
@@ -15796,7 +16004,9 @@
       <c r="F256" t="n">
         <v>38</v>
       </c>
-      <c r="G256" t="inlineStr"/>
+      <c r="G256" t="n">
+        <v>12</v>
+      </c>
       <c r="H256" t="n">
         <v>9</v>
       </c>
@@ -15830,7 +16040,9 @@
       <c r="R256" t="n">
         <v>22.22222222222222</v>
       </c>
-      <c r="S256" t="inlineStr"/>
+      <c r="S256" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="257">
       <c r="A257" t="n">
@@ -15958,7 +16170,9 @@
       <c r="A259" t="n">
         <v>280</v>
       </c>
-      <c r="B259" t="inlineStr"/>
+      <c r="B259" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C259" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -16000,11 +16214,15 @@
       <c r="O259" t="n">
         <v>1</v>
       </c>
-      <c r="P259" t="inlineStr"/>
+      <c r="P259" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q259" t="n">
         <v>0.3026436494672071</v>
       </c>
-      <c r="R259" t="inlineStr"/>
+      <c r="R259" t="n">
+        <v>18.19</v>
+      </c>
       <c r="S259" t="n">
         <v>0.8</v>
       </c>
@@ -16946,7 +17164,9 @@
       <c r="G275" t="n">
         <v>12</v>
       </c>
-      <c r="H275" t="inlineStr"/>
+      <c r="H275" t="n">
+        <v>11</v>
+      </c>
       <c r="I275" t="n">
         <v>2</v>
       </c>
@@ -16977,7 +17197,9 @@
       <c r="R275" t="n">
         <v>7.090909090909091</v>
       </c>
-      <c r="S275" t="inlineStr"/>
+      <c r="S275" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="276">
       <c r="A276" t="n">
@@ -17000,7 +17222,9 @@
       <c r="F276" t="n">
         <v>45</v>
       </c>
-      <c r="G276" t="inlineStr"/>
+      <c r="G276" t="n">
+        <v>12</v>
+      </c>
       <c r="H276" t="n">
         <v>22</v>
       </c>
@@ -17034,7 +17258,9 @@
       <c r="R276" t="n">
         <v>27.5</v>
       </c>
-      <c r="S276" t="inlineStr"/>
+      <c r="S276" t="n">
+        <v>0.5217391304347826</v>
+      </c>
     </row>
     <row r="277">
       <c r="A277" t="n">
@@ -17081,7 +17307,9 @@
       <c r="N277" t="n">
         <v>1</v>
       </c>
-      <c r="O277" t="inlineStr"/>
+      <c r="O277" t="n">
+        <v>2</v>
+      </c>
       <c r="P277" t="n">
         <v>0.4394980579623544</v>
       </c>
@@ -17116,7 +17344,9 @@
       <c r="F278" t="n">
         <v>38</v>
       </c>
-      <c r="G278" t="inlineStr"/>
+      <c r="G278" t="n">
+        <v>12</v>
+      </c>
       <c r="H278" t="n">
         <v>5</v>
       </c>
@@ -17150,7 +17380,9 @@
       <c r="R278" t="n">
         <v>22.21666666666667</v>
       </c>
-      <c r="S278" t="inlineStr"/>
+      <c r="S278" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="279">
       <c r="A279" t="n">
@@ -17644,7 +17876,9 @@
       <c r="A287" t="n">
         <v>308</v>
       </c>
-      <c r="B287" t="inlineStr"/>
+      <c r="B287" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C287" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -17686,11 +17920,15 @@
       <c r="O287" t="n">
         <v>0</v>
       </c>
-      <c r="P287" t="inlineStr"/>
+      <c r="P287" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q287" t="n">
         <v>1.088613724202939</v>
       </c>
-      <c r="R287" t="inlineStr"/>
+      <c r="R287" t="n">
+        <v>18.94791666666667</v>
+      </c>
       <c r="S287" t="n">
         <v>1.285714285714286</v>
       </c>
@@ -17838,7 +18076,9 @@
       <c r="F290" t="n">
         <v>42</v>
       </c>
-      <c r="G290" t="inlineStr"/>
+      <c r="G290" t="n">
+        <v>12</v>
+      </c>
       <c r="H290" t="n">
         <v>10</v>
       </c>
@@ -17872,7 +18112,9 @@
       <c r="R290" t="n">
         <v>20.3</v>
       </c>
-      <c r="S290" t="inlineStr"/>
+      <c r="S290" t="n">
+        <v>1.090909090909091</v>
+      </c>
     </row>
     <row r="291">
       <c r="A291" t="n">
@@ -18133,7 +18375,9 @@
       <c r="D295" t="n">
         <v>40</v>
       </c>
-      <c r="E295" t="inlineStr"/>
+      <c r="E295" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F295" t="n">
         <v>26</v>
       </c>
@@ -18213,7 +18457,9 @@
       <c r="K296" t="n">
         <v>1</v>
       </c>
-      <c r="L296" t="inlineStr"/>
+      <c r="L296" t="n">
+        <v>0</v>
+      </c>
       <c r="M296" t="n">
         <v>1</v>
       </c>
@@ -18789,7 +19035,9 @@
       <c r="A306" t="n">
         <v>330</v>
       </c>
-      <c r="B306" t="inlineStr"/>
+      <c r="B306" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C306" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -18831,11 +19079,15 @@
       <c r="O306" t="n">
         <v>2</v>
       </c>
-      <c r="P306" t="inlineStr"/>
+      <c r="P306" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q306" t="n">
         <v>1.219608736658895</v>
       </c>
-      <c r="R306" t="inlineStr"/>
+      <c r="R306" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S306" t="n">
         <v>1.777777777777778</v>
       </c>
@@ -18998,7 +19250,9 @@
       <c r="K309" t="n">
         <v>1</v>
       </c>
-      <c r="L309" t="inlineStr"/>
+      <c r="L309" t="n">
+        <v>0</v>
+      </c>
       <c r="M309" t="n">
         <v>1</v>
       </c>
@@ -19066,7 +19320,9 @@
       <c r="N310" t="n">
         <v>1</v>
       </c>
-      <c r="O310" t="inlineStr"/>
+      <c r="O310" t="n">
+        <v>2</v>
+      </c>
       <c r="P310" t="n">
         <v>0.3970720047804003</v>
       </c>
@@ -19360,7 +19616,9 @@
       <c r="K315" t="n">
         <v>1</v>
       </c>
-      <c r="L315" t="inlineStr"/>
+      <c r="L315" t="n">
+        <v>0</v>
+      </c>
       <c r="M315" t="n">
         <v>0</v>
       </c>
@@ -19507,7 +19765,9 @@
       <c r="A318" t="n">
         <v>343</v>
       </c>
-      <c r="B318" t="inlineStr"/>
+      <c r="B318" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C318" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -19549,11 +19809,15 @@
       <c r="O318" t="n">
         <v>3</v>
       </c>
-      <c r="P318" t="inlineStr"/>
+      <c r="P318" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q318" t="n">
         <v>-0.7453164501804357</v>
       </c>
-      <c r="R318" t="inlineStr"/>
+      <c r="R318" t="n">
+        <v>20.21111111111111</v>
+      </c>
       <c r="S318" t="n">
         <v>1.444444444444444</v>
       </c>
@@ -19777,7 +20041,9 @@
       <c r="K322" t="n">
         <v>1</v>
       </c>
-      <c r="L322" t="inlineStr"/>
+      <c r="L322" t="n">
+        <v>0</v>
+      </c>
       <c r="M322" t="n">
         <v>0</v>
       </c>
@@ -20231,7 +20497,9 @@
       <c r="A330" t="n">
         <v>355</v>
       </c>
-      <c r="B330" t="inlineStr"/>
+      <c r="B330" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C330" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -20273,11 +20541,15 @@
       <c r="O330" t="n">
         <v>4</v>
       </c>
-      <c r="P330" t="inlineStr"/>
+      <c r="P330" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q330" t="n">
         <v>-0.6143214377244803</v>
       </c>
-      <c r="R330" t="inlineStr"/>
+      <c r="R330" t="n">
+        <v>18.19</v>
+      </c>
       <c r="S330" t="n">
         <v>0.9285714285714286</v>
       </c>
@@ -20286,7 +20558,9 @@
       <c r="A331" t="n">
         <v>356</v>
       </c>
-      <c r="B331" t="inlineStr"/>
+      <c r="B331" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C331" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -20328,11 +20602,15 @@
       <c r="O331" t="n">
         <v>3</v>
       </c>
-      <c r="P331" t="inlineStr"/>
+      <c r="P331" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q331" t="n">
         <v>0.8266236992910285</v>
       </c>
-      <c r="R331" t="inlineStr"/>
+      <c r="R331" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S331" t="n">
         <v>1.2</v>
       </c>
@@ -20341,7 +20619,9 @@
       <c r="A332" t="n">
         <v>358</v>
       </c>
-      <c r="B332" t="inlineStr"/>
+      <c r="B332" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C332" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -20383,11 +20663,15 @@
       <c r="O332" t="n">
         <v>5</v>
       </c>
-      <c r="P332" t="inlineStr"/>
+      <c r="P332" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q332" t="n">
         <v>0.4336386619231625</v>
       </c>
-      <c r="R332" t="inlineStr"/>
+      <c r="R332" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S332" t="n">
         <v>1.714285714285714</v>
       </c>
@@ -20396,7 +20680,9 @@
       <c r="A333" t="n">
         <v>359</v>
       </c>
-      <c r="B333" t="inlineStr"/>
+      <c r="B333" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C333" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -20438,11 +20724,15 @@
       <c r="O333" t="n">
         <v>0</v>
       </c>
-      <c r="P333" t="inlineStr"/>
+      <c r="P333" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q333" t="n">
         <v>0.9576187117469839</v>
       </c>
-      <c r="R333" t="inlineStr"/>
+      <c r="R333" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S333" t="n">
         <v>0.5714285714285714</v>
       </c>
@@ -20451,7 +20741,9 @@
       <c r="A334" t="n">
         <v>360</v>
       </c>
-      <c r="B334" t="inlineStr"/>
+      <c r="B334" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C334" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -20493,11 +20785,15 @@
       <c r="O334" t="n">
         <v>5</v>
       </c>
-      <c r="P334" t="inlineStr"/>
+      <c r="P334" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q334" t="n">
         <v>0.04065362455529643</v>
       </c>
-      <c r="R334" t="inlineStr"/>
+      <c r="R334" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S334" t="n">
         <v>1.555555555555556</v>
       </c>
@@ -20523,7 +20819,9 @@
       <c r="F335" t="n">
         <v>36</v>
       </c>
-      <c r="G335" t="inlineStr"/>
+      <c r="G335" t="n">
+        <v>12</v>
+      </c>
       <c r="H335" t="n">
         <v>9</v>
       </c>
@@ -20557,7 +20855,9 @@
       <c r="R335" t="n">
         <v>28.97777777777778</v>
       </c>
-      <c r="S335" t="inlineStr"/>
+      <c r="S335" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="336">
       <c r="A336" t="n">
@@ -20644,7 +20944,9 @@
       <c r="G337" t="n">
         <v>12</v>
       </c>
-      <c r="H337" t="inlineStr"/>
+      <c r="H337" t="n">
+        <v>11</v>
+      </c>
       <c r="I337" t="n">
         <v>16</v>
       </c>
@@ -20675,7 +20977,9 @@
       <c r="R337" t="n">
         <v>22.275</v>
       </c>
-      <c r="S337" t="inlineStr"/>
+      <c r="S337" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="338">
       <c r="A338" t="n">
@@ -20881,7 +21185,9 @@
       <c r="F341" t="n">
         <v>45</v>
       </c>
-      <c r="G341" t="inlineStr"/>
+      <c r="G341" t="n">
+        <v>12</v>
+      </c>
       <c r="H341" t="n">
         <v>16</v>
       </c>
@@ -20915,7 +21221,9 @@
       <c r="R341" t="n">
         <v>12.5</v>
       </c>
-      <c r="S341" t="inlineStr"/>
+      <c r="S341" t="n">
+        <v>0.7058823529411765</v>
+      </c>
     </row>
     <row r="342">
       <c r="A342" t="n">
@@ -21084,7 +21392,9 @@
       <c r="N344" t="n">
         <v>1</v>
       </c>
-      <c r="O344" t="inlineStr"/>
+      <c r="O344" t="n">
+        <v>2</v>
+      </c>
       <c r="P344" t="n">
         <v>0.5162832387212428</v>
       </c>
@@ -21285,7 +21595,9 @@
       <c r="A348" t="n">
         <v>375</v>
       </c>
-      <c r="B348" t="inlineStr"/>
+      <c r="B348" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C348" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -21327,11 +21639,15 @@
       <c r="O348" t="n">
         <v>2</v>
       </c>
-      <c r="P348" t="inlineStr"/>
+      <c r="P348" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q348" t="n">
         <v>1.219608736658895</v>
       </c>
-      <c r="R348" t="inlineStr"/>
+      <c r="R348" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S348" t="n">
         <v>0.9285714285714286</v>
       </c>
@@ -21665,7 +21981,9 @@
       <c r="G354" t="n">
         <v>13</v>
       </c>
-      <c r="H354" t="inlineStr"/>
+      <c r="H354" t="n">
+        <v>11</v>
+      </c>
       <c r="I354" t="n">
         <v>1</v>
       </c>
@@ -21696,7 +22014,9 @@
       <c r="R354" t="n">
         <v>18.625</v>
       </c>
-      <c r="S354" t="inlineStr"/>
+      <c r="S354" t="n">
+        <v>1.083333333333333</v>
+      </c>
     </row>
     <row r="355">
       <c r="A355" t="n">
@@ -22125,7 +22445,9 @@
       <c r="A362" t="n">
         <v>389</v>
       </c>
-      <c r="B362" t="inlineStr"/>
+      <c r="B362" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C362" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -22167,11 +22489,15 @@
       <c r="O362" t="n">
         <v>2</v>
       </c>
-      <c r="P362" t="inlineStr"/>
+      <c r="P362" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q362" t="n">
         <v>-0.7453164501804357</v>
       </c>
-      <c r="R362" t="inlineStr"/>
+      <c r="R362" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S362" t="n">
         <v>1.272727272727273</v>
       </c>
@@ -22322,7 +22648,9 @@
       <c r="G365" t="n">
         <v>17</v>
       </c>
-      <c r="H365" t="inlineStr"/>
+      <c r="H365" t="n">
+        <v>11</v>
+      </c>
       <c r="I365" t="n">
         <v>13</v>
       </c>
@@ -22353,7 +22681,9 @@
       <c r="R365" t="n">
         <v>13.08</v>
       </c>
-      <c r="S365" t="inlineStr"/>
+      <c r="S365" t="n">
+        <v>1.416666666666667</v>
+      </c>
     </row>
     <row r="366">
       <c r="A366" t="n">
@@ -22418,7 +22748,9 @@
       <c r="A367" t="n">
         <v>394</v>
       </c>
-      <c r="B367" t="inlineStr"/>
+      <c r="B367" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C367" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -22460,11 +22792,15 @@
       <c r="O367" t="n">
         <v>4</v>
       </c>
-      <c r="P367" t="inlineStr"/>
+      <c r="P367" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q367" t="n">
         <v>-1.531286524916168</v>
       </c>
-      <c r="R367" t="inlineStr"/>
+      <c r="R367" t="n">
+        <v>21.15116279069768</v>
+      </c>
       <c r="S367" t="n">
         <v>0.8</v>
       </c>
@@ -22490,7 +22826,9 @@
       <c r="F368" t="n">
         <v>41</v>
       </c>
-      <c r="G368" t="inlineStr"/>
+      <c r="G368" t="n">
+        <v>12</v>
+      </c>
       <c r="H368" t="n">
         <v>8</v>
       </c>
@@ -22524,7 +22862,9 @@
       <c r="R368" t="n">
         <v>22.72727272727273</v>
       </c>
-      <c r="S368" t="inlineStr"/>
+      <c r="S368" t="n">
+        <v>1.333333333333333</v>
+      </c>
     </row>
     <row r="369">
       <c r="A369" t="n">
@@ -22562,7 +22902,9 @@
       <c r="K369" t="n">
         <v>1</v>
       </c>
-      <c r="L369" t="inlineStr"/>
+      <c r="L369" t="n">
+        <v>0</v>
+      </c>
       <c r="M369" t="n">
         <v>0</v>
       </c>
@@ -22589,7 +22931,9 @@
       <c r="A370" t="n">
         <v>397</v>
       </c>
-      <c r="B370" t="inlineStr"/>
+      <c r="B370" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C370" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -22631,11 +22975,15 @@
       <c r="O370" t="n">
         <v>4</v>
       </c>
-      <c r="P370" t="inlineStr"/>
+      <c r="P370" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q370" t="n">
         <v>0.3026436494672071</v>
       </c>
-      <c r="R370" t="inlineStr"/>
+      <c r="R370" t="n">
+        <v>18.19</v>
+      </c>
       <c r="S370" t="n">
         <v>0.631578947368421</v>
       </c>
@@ -22827,7 +23175,9 @@
       <c r="A374" t="n">
         <v>401</v>
       </c>
-      <c r="B374" t="inlineStr"/>
+      <c r="B374" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C374" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -22869,11 +23219,15 @@
       <c r="O374" t="n">
         <v>7</v>
       </c>
-      <c r="P374" t="inlineStr"/>
+      <c r="P374" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q374" t="n">
         <v>-0.483326425268525</v>
       </c>
-      <c r="R374" t="inlineStr"/>
+      <c r="R374" t="n">
+        <v>13.99230769230769</v>
+      </c>
       <c r="S374" t="n">
         <v>1</v>
       </c>
@@ -22963,7 +23317,9 @@
       <c r="G376" t="n">
         <v>12</v>
       </c>
-      <c r="H376" t="inlineStr"/>
+      <c r="H376" t="n">
+        <v>11</v>
+      </c>
       <c r="I376" t="n">
         <v>4</v>
       </c>
@@ -22994,7 +23350,9 @@
       <c r="R376" t="n">
         <v>11.125</v>
       </c>
-      <c r="S376" t="inlineStr"/>
+      <c r="S376" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="377">
       <c r="A377" t="n">
@@ -23142,7 +23500,9 @@
       <c r="G379" t="n">
         <v>12</v>
       </c>
-      <c r="H379" t="inlineStr"/>
+      <c r="H379" t="n">
+        <v>11</v>
+      </c>
       <c r="I379" t="n">
         <v>7</v>
       </c>
@@ -23173,7 +23533,9 @@
       <c r="R379" t="n">
         <v>34.375</v>
       </c>
-      <c r="S379" t="inlineStr"/>
+      <c r="S379" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="380">
       <c r="A380" t="n">
@@ -23190,7 +23552,9 @@
       <c r="D380" t="n">
         <v>40</v>
       </c>
-      <c r="E380" t="inlineStr"/>
+      <c r="E380" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F380" t="n">
         <v>44</v>
       </c>
@@ -23563,7 +23927,9 @@
       <c r="G386" t="n">
         <v>14</v>
       </c>
-      <c r="H386" t="inlineStr"/>
+      <c r="H386" t="n">
+        <v>11</v>
+      </c>
       <c r="I386" t="n">
         <v>4</v>
       </c>
@@ -23594,7 +23960,9 @@
       <c r="R386" t="n">
         <v>28.48</v>
       </c>
-      <c r="S386" t="inlineStr"/>
+      <c r="S386" t="n">
+        <v>1.166666666666667</v>
+      </c>
     </row>
     <row r="387">
       <c r="A387" t="n">
@@ -23794,7 +24162,9 @@
       <c r="D390" t="n">
         <v>50</v>
       </c>
-      <c r="E390" t="inlineStr"/>
+      <c r="E390" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F390" t="n">
         <v>31</v>
       </c>
@@ -23964,7 +24334,9 @@
       <c r="A393" t="n">
         <v>420</v>
       </c>
-      <c r="B393" t="inlineStr"/>
+      <c r="B393" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C393" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -24006,11 +24378,15 @@
       <c r="O393" t="n">
         <v>1</v>
       </c>
-      <c r="P393" t="inlineStr"/>
+      <c r="P393" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q393" t="n">
         <v>1.35060374911485</v>
       </c>
-      <c r="R393" t="inlineStr"/>
+      <c r="R393" t="n">
+        <v>16.53636363636364</v>
+      </c>
       <c r="S393" t="n">
         <v>2.6</v>
       </c>
@@ -24036,7 +24412,9 @@
       <c r="F394" t="n">
         <v>29</v>
       </c>
-      <c r="G394" t="inlineStr"/>
+      <c r="G394" t="n">
+        <v>12</v>
+      </c>
       <c r="H394" t="n">
         <v>16</v>
       </c>
@@ -24070,7 +24448,9 @@
       <c r="R394" t="n">
         <v>17.08888888888889</v>
       </c>
-      <c r="S394" t="inlineStr"/>
+      <c r="S394" t="n">
+        <v>0.7058823529411765</v>
+      </c>
     </row>
     <row r="395">
       <c r="A395" t="n">
@@ -24645,7 +25025,9 @@
       <c r="G404" t="n">
         <v>16</v>
       </c>
-      <c r="H404" t="inlineStr"/>
+      <c r="H404" t="n">
+        <v>11</v>
+      </c>
       <c r="I404" t="n">
         <v>2</v>
       </c>
@@ -24676,7 +25058,9 @@
       <c r="R404" t="n">
         <v>13.9</v>
       </c>
-      <c r="S404" t="inlineStr"/>
+      <c r="S404" t="n">
+        <v>1.333333333333333</v>
+      </c>
     </row>
     <row r="405">
       <c r="A405" t="n">
@@ -24937,7 +25321,9 @@
       <c r="D409" t="n">
         <v>42</v>
       </c>
-      <c r="E409" t="inlineStr"/>
+      <c r="E409" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F409" t="n">
         <v>28</v>
       </c>
@@ -25046,7 +25432,9 @@
       <c r="A411" t="n">
         <v>439</v>
       </c>
-      <c r="B411" t="inlineStr"/>
+      <c r="B411" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C411" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -25088,11 +25476,15 @@
       <c r="O411" t="n">
         <v>2</v>
       </c>
-      <c r="P411" t="inlineStr"/>
+      <c r="P411" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q411" t="n">
         <v>0.6956286868350732</v>
       </c>
-      <c r="R411" t="inlineStr"/>
+      <c r="R411" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S411" t="n">
         <v>0.9230769230769231</v>
       </c>
@@ -25173,7 +25565,9 @@
       <c r="D413" t="n">
         <v>40</v>
       </c>
-      <c r="E413" t="inlineStr"/>
+      <c r="E413" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F413" t="n">
         <v>31</v>
       </c>
@@ -25465,7 +25859,9 @@
       <c r="A418" t="n">
         <v>447</v>
       </c>
-      <c r="B418" t="inlineStr"/>
+      <c r="B418" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C418" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -25507,11 +25903,15 @@
       <c r="O418" t="n">
         <v>3</v>
       </c>
-      <c r="P418" t="inlineStr"/>
+      <c r="P418" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q418" t="n">
         <v>1.088613724202939</v>
       </c>
-      <c r="R418" t="inlineStr"/>
+      <c r="R418" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S418" t="n">
         <v>2.6</v>
       </c>
@@ -25674,7 +26074,9 @@
       <c r="K421" t="n">
         <v>1</v>
       </c>
-      <c r="L421" t="inlineStr"/>
+      <c r="L421" t="n">
+        <v>0</v>
+      </c>
       <c r="M421" t="n">
         <v>0</v>
       </c>
@@ -25962,7 +26364,9 @@
       <c r="F426" t="n">
         <v>48</v>
       </c>
-      <c r="G426" t="inlineStr"/>
+      <c r="G426" t="n">
+        <v>12</v>
+      </c>
       <c r="H426" t="n">
         <v>15</v>
       </c>
@@ -25996,7 +26400,9 @@
       <c r="R426" t="n">
         <v>37.21621621621622</v>
       </c>
-      <c r="S426" t="inlineStr"/>
+      <c r="S426" t="n">
+        <v>0.75</v>
+      </c>
     </row>
     <row r="427">
       <c r="A427" t="n">
@@ -26074,7 +26480,9 @@
       <c r="D428" t="n">
         <v>43</v>
       </c>
-      <c r="E428" t="inlineStr"/>
+      <c r="E428" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F428" t="n">
         <v>28</v>
       </c>
@@ -26459,7 +26867,9 @@
       <c r="K434" t="n">
         <v>1</v>
       </c>
-      <c r="L434" t="inlineStr"/>
+      <c r="L434" t="n">
+        <v>0</v>
+      </c>
       <c r="M434" t="n">
         <v>0</v>
       </c>
@@ -26891,7 +27301,9 @@
       <c r="N441" t="n">
         <v>1</v>
       </c>
-      <c r="O441" t="inlineStr"/>
+      <c r="O441" t="n">
+        <v>2</v>
+      </c>
       <c r="P441" t="n">
         <v>0.3023603226770242</v>
       </c>
@@ -27292,7 +27704,9 @@
       <c r="F448" t="n">
         <v>37</v>
       </c>
-      <c r="G448" t="inlineStr"/>
+      <c r="G448" t="n">
+        <v>12</v>
+      </c>
       <c r="H448" t="n">
         <v>16</v>
       </c>
@@ -27326,7 +27740,9 @@
       <c r="R448" t="n">
         <v>8.65</v>
       </c>
-      <c r="S448" t="inlineStr"/>
+      <c r="S448" t="n">
+        <v>0.7058823529411765</v>
+      </c>
     </row>
     <row r="449">
       <c r="A449" t="n">
@@ -27593,7 +28009,9 @@
       <c r="F453" t="n">
         <v>42</v>
       </c>
-      <c r="G453" t="inlineStr"/>
+      <c r="G453" t="n">
+        <v>12</v>
+      </c>
       <c r="H453" t="n">
         <v>19</v>
       </c>
@@ -27627,7 +28045,9 @@
       <c r="R453" t="n">
         <v>22.1</v>
       </c>
-      <c r="S453" t="inlineStr"/>
+      <c r="S453" t="n">
+        <v>0.6</v>
+      </c>
     </row>
     <row r="454">
       <c r="A454" t="n">
@@ -27894,7 +28314,9 @@
       <c r="F458" t="n">
         <v>23</v>
       </c>
-      <c r="G458" t="inlineStr"/>
+      <c r="G458" t="n">
+        <v>12</v>
+      </c>
       <c r="H458" t="n">
         <v>11</v>
       </c>
@@ -27928,7 +28350,9 @@
       <c r="R458" t="n">
         <v>11.20408163265306</v>
       </c>
-      <c r="S458" t="inlineStr"/>
+      <c r="S458" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="459">
       <c r="A459" t="n">
@@ -28422,7 +28846,9 @@
       <c r="A467" t="n">
         <v>502</v>
       </c>
-      <c r="B467" t="inlineStr"/>
+      <c r="B467" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C467" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -28464,11 +28890,15 @@
       <c r="O467" t="n">
         <v>13</v>
       </c>
-      <c r="P467" t="inlineStr"/>
+      <c r="P467" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q467" t="n">
         <v>-1.531286524916168</v>
       </c>
-      <c r="R467" t="inlineStr"/>
+      <c r="R467" t="n">
+        <v>20.21111111111111</v>
+      </c>
       <c r="S467" t="n">
         <v>1.1</v>
       </c>
@@ -28823,7 +29253,9 @@
       <c r="N473" t="n">
         <v>0</v>
       </c>
-      <c r="O473" t="inlineStr"/>
+      <c r="O473" t="n">
+        <v>2</v>
+      </c>
       <c r="P473" t="n">
         <v>0.2195996414699731</v>
       </c>
@@ -29695,7 +30127,9 @@
       <c r="A488" t="n">
         <v>524</v>
       </c>
-      <c r="B488" t="inlineStr"/>
+      <c r="B488" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C488" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -29737,11 +30171,15 @@
       <c r="O488" t="n">
         <v>7</v>
       </c>
-      <c r="P488" t="inlineStr"/>
+      <c r="P488" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q488" t="n">
         <v>-0.09034138790065893</v>
       </c>
-      <c r="R488" t="inlineStr"/>
+      <c r="R488" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S488" t="n">
         <v>2.25</v>
       </c>
@@ -29892,7 +30330,9 @@
       <c r="G491" t="n">
         <v>17</v>
       </c>
-      <c r="H491" t="inlineStr"/>
+      <c r="H491" t="n">
+        <v>11</v>
+      </c>
       <c r="I491" t="n">
         <v>9</v>
       </c>
@@ -29923,7 +30363,9 @@
       <c r="R491" t="n">
         <v>33.22222222222222</v>
       </c>
-      <c r="S491" t="inlineStr"/>
+      <c r="S491" t="n">
+        <v>1.416666666666667</v>
+      </c>
     </row>
     <row r="492">
       <c r="A492" t="n">
@@ -29990,7 +30432,9 @@
       <c r="A493" t="n">
         <v>531</v>
       </c>
-      <c r="B493" t="inlineStr"/>
+      <c r="B493" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C493" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -30032,11 +30476,15 @@
       <c r="O493" t="n">
         <v>2</v>
       </c>
-      <c r="P493" t="inlineStr"/>
+      <c r="P493" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q493" t="n">
         <v>-0.09034138790065893</v>
       </c>
-      <c r="R493" t="inlineStr"/>
+      <c r="R493" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S493" t="n">
         <v>1.857142857142857</v>
       </c>
@@ -30245,7 +30693,9 @@
       <c r="F497" t="n">
         <v>48</v>
       </c>
-      <c r="G497" t="inlineStr"/>
+      <c r="G497" t="n">
+        <v>12</v>
+      </c>
       <c r="H497" t="n">
         <v>16</v>
       </c>
@@ -30279,7 +30729,9 @@
       <c r="R497" t="n">
         <v>53.425</v>
       </c>
-      <c r="S497" t="inlineStr"/>
+      <c r="S497" t="n">
+        <v>0.7058823529411765</v>
+      </c>
     </row>
     <row r="498">
       <c r="A498" t="n">
@@ -31198,7 +31650,9 @@
       <c r="A513" t="n">
         <v>551</v>
       </c>
-      <c r="B513" t="inlineStr"/>
+      <c r="B513" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C513" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -31240,11 +31694,15 @@
       <c r="O513" t="n">
         <v>1</v>
       </c>
-      <c r="P513" t="inlineStr"/>
+      <c r="P513" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q513" t="n">
         <v>0.3026436494672071</v>
       </c>
-      <c r="R513" t="inlineStr"/>
+      <c r="R513" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S513" t="n">
         <v>1</v>
       </c>
@@ -31434,7 +31892,9 @@
       <c r="A517" t="n">
         <v>557</v>
       </c>
-      <c r="B517" t="inlineStr"/>
+      <c r="B517" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C517" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -31476,11 +31936,15 @@
       <c r="O517" t="n">
         <v>9</v>
       </c>
-      <c r="P517" t="inlineStr"/>
+      <c r="P517" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q517" t="n">
         <v>-0.6143214377244803</v>
       </c>
-      <c r="R517" t="inlineStr"/>
+      <c r="R517" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S517" t="n">
         <v>0.4166666666666667</v>
       </c>
@@ -31591,7 +32055,9 @@
       <c r="N519" t="n">
         <v>0</v>
       </c>
-      <c r="O519" t="inlineStr"/>
+      <c r="O519" t="n">
+        <v>2</v>
+      </c>
       <c r="P519" t="n">
         <v>0.09859575739468179</v>
       </c>
@@ -31626,7 +32092,9 @@
       <c r="F520" t="n">
         <v>28</v>
       </c>
-      <c r="G520" t="inlineStr"/>
+      <c r="G520" t="n">
+        <v>12</v>
+      </c>
       <c r="H520" t="n">
         <v>13</v>
       </c>
@@ -31660,7 +32128,9 @@
       <c r="R520" t="n">
         <v>39.375</v>
       </c>
-      <c r="S520" t="inlineStr"/>
+      <c r="S520" t="n">
+        <v>0.8571428571428571</v>
+      </c>
     </row>
     <row r="521">
       <c r="A521" t="n">
@@ -31869,7 +32339,9 @@
       <c r="G524" t="n">
         <v>18</v>
       </c>
-      <c r="H524" t="inlineStr"/>
+      <c r="H524" t="n">
+        <v>11</v>
+      </c>
       <c r="I524" t="n">
         <v>2</v>
       </c>
@@ -31900,7 +32372,9 @@
       <c r="R524" t="n">
         <v>27.68</v>
       </c>
-      <c r="S524" t="inlineStr"/>
+      <c r="S524" t="n">
+        <v>1.5</v>
+      </c>
     </row>
     <row r="525">
       <c r="A525" t="n">
@@ -31917,7 +32391,9 @@
       <c r="D525" t="n">
         <v>40</v>
       </c>
-      <c r="E525" t="inlineStr"/>
+      <c r="E525" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F525" t="n">
         <v>42</v>
       </c>
@@ -32424,7 +32900,9 @@
       <c r="K533" t="n">
         <v>1</v>
       </c>
-      <c r="L533" t="inlineStr"/>
+      <c r="L533" t="n">
+        <v>0</v>
+      </c>
       <c r="M533" t="n">
         <v>0</v>
       </c>
@@ -32471,7 +32949,9 @@
       <c r="G534" t="n">
         <v>12</v>
       </c>
-      <c r="H534" t="inlineStr"/>
+      <c r="H534" t="n">
+        <v>11</v>
+      </c>
       <c r="I534" t="n">
         <v>10</v>
       </c>
@@ -32502,7 +32982,9 @@
       <c r="R534" t="n">
         <v>12.375</v>
       </c>
-      <c r="S534" t="inlineStr"/>
+      <c r="S534" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="535">
       <c r="A535" t="n">
@@ -32647,7 +33129,9 @@
       <c r="F537" t="n">
         <v>49</v>
       </c>
-      <c r="G537" t="inlineStr"/>
+      <c r="G537" t="n">
+        <v>12</v>
+      </c>
       <c r="H537" t="n">
         <v>9</v>
       </c>
@@ -32681,7 +33165,9 @@
       <c r="R537" t="n">
         <v>13.84</v>
       </c>
-      <c r="S537" t="inlineStr"/>
+      <c r="S537" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="538">
       <c r="A538" t="n">
@@ -32748,7 +33234,9 @@
       <c r="A539" t="n">
         <v>583</v>
       </c>
-      <c r="B539" t="inlineStr"/>
+      <c r="B539" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C539" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -32790,11 +33278,15 @@
       <c r="O539" t="n">
         <v>2</v>
       </c>
-      <c r="P539" t="inlineStr"/>
+      <c r="P539" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q539" t="n">
         <v>-0.7453164501804357</v>
       </c>
-      <c r="R539" t="inlineStr"/>
+      <c r="R539" t="n">
+        <v>18.94791666666667</v>
+      </c>
       <c r="S539" t="n">
         <v>2</v>
       </c>
@@ -32881,7 +33373,9 @@
       <c r="F541" t="n">
         <v>22</v>
       </c>
-      <c r="G541" t="inlineStr"/>
+      <c r="G541" t="n">
+        <v>12</v>
+      </c>
       <c r="H541" t="n">
         <v>10</v>
       </c>
@@ -32915,7 +33409,9 @@
       <c r="R541" t="n">
         <v>15.5</v>
       </c>
-      <c r="S541" t="inlineStr"/>
+      <c r="S541" t="n">
+        <v>1.090909090909091</v>
+      </c>
     </row>
     <row r="542">
       <c r="A542" t="n">
@@ -33670,7 +34166,9 @@
       <c r="F554" t="n">
         <v>32</v>
       </c>
-      <c r="G554" t="inlineStr"/>
+      <c r="G554" t="n">
+        <v>12</v>
+      </c>
       <c r="H554" t="n">
         <v>18</v>
       </c>
@@ -33704,7 +34202,9 @@
       <c r="R554" t="n">
         <v>15.625</v>
       </c>
-      <c r="S554" t="inlineStr"/>
+      <c r="S554" t="n">
+        <v>0.631578947368421</v>
+      </c>
     </row>
     <row r="555">
       <c r="A555" t="n">
@@ -33742,7 +34242,9 @@
       <c r="K555" t="n">
         <v>1</v>
       </c>
-      <c r="L555" t="inlineStr"/>
+      <c r="L555" t="n">
+        <v>0</v>
+      </c>
       <c r="M555" t="n">
         <v>0</v>
       </c>
@@ -33900,7 +34402,9 @@
       <c r="D558" t="n">
         <v>40</v>
       </c>
-      <c r="E558" t="inlineStr"/>
+      <c r="E558" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F558" t="n">
         <v>27</v>
       </c>
@@ -34375,7 +34879,9 @@
       <c r="A566" t="n">
         <v>613</v>
       </c>
-      <c r="B566" t="inlineStr"/>
+      <c r="B566" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C566" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -34417,11 +34923,15 @@
       <c r="O566" t="n">
         <v>2</v>
       </c>
-      <c r="P566" t="inlineStr"/>
+      <c r="P566" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q566" t="n">
         <v>0.04065362455529643</v>
       </c>
-      <c r="R566" t="inlineStr"/>
+      <c r="R566" t="n">
+        <v>18.19</v>
+      </c>
       <c r="S566" t="n">
         <v>0.8235294117647058</v>
       </c>
@@ -34430,7 +34940,9 @@
       <c r="A567" t="n">
         <v>614</v>
       </c>
-      <c r="B567" t="inlineStr"/>
+      <c r="B567" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C567" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -34472,11 +34984,15 @@
       <c r="O567" t="n">
         <v>3</v>
       </c>
-      <c r="P567" t="inlineStr"/>
+      <c r="P567" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q567" t="n">
         <v>0.4336386619231625</v>
       </c>
-      <c r="R567" t="inlineStr"/>
+      <c r="R567" t="n">
+        <v>18.19</v>
+      </c>
       <c r="S567" t="n">
         <v>0.875</v>
       </c>
@@ -34790,7 +35306,9 @@
       <c r="A573" t="n">
         <v>620</v>
       </c>
-      <c r="B573" t="inlineStr"/>
+      <c r="B573" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C573" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -34832,11 +35350,15 @@
       <c r="O573" t="n">
         <v>7</v>
       </c>
-      <c r="P573" t="inlineStr"/>
+      <c r="P573" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q573" t="n">
         <v>-0.483326425268525</v>
       </c>
-      <c r="R573" t="inlineStr"/>
+      <c r="R573" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S573" t="n">
         <v>1.181818181818182</v>
       </c>
@@ -35039,7 +35561,9 @@
       <c r="D577" t="n">
         <v>45</v>
       </c>
-      <c r="E577" t="inlineStr"/>
+      <c r="E577" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F577" t="n">
         <v>46</v>
       </c>
@@ -35485,7 +36009,9 @@
       <c r="K584" t="n">
         <v>1</v>
       </c>
-      <c r="L584" t="inlineStr"/>
+      <c r="L584" t="n">
+        <v>0</v>
+      </c>
       <c r="M584" t="n">
         <v>1</v>
       </c>
@@ -35645,7 +36171,9 @@
       <c r="D587" t="n">
         <v>40</v>
       </c>
-      <c r="E587" t="inlineStr"/>
+      <c r="E587" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F587" t="n">
         <v>55</v>
       </c>
@@ -35734,7 +36262,9 @@
       <c r="N588" t="n">
         <v>0</v>
       </c>
-      <c r="O588" t="inlineStr"/>
+      <c r="O588" t="n">
+        <v>2</v>
+      </c>
       <c r="P588" t="n">
         <v>0.2037645652823424</v>
       </c>
@@ -36299,7 +36829,9 @@
       <c r="A598" t="n">
         <v>648</v>
       </c>
-      <c r="B598" t="inlineStr"/>
+      <c r="B598" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C598" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -36341,11 +36873,15 @@
       <c r="O598" t="n">
         <v>1</v>
       </c>
-      <c r="P598" t="inlineStr"/>
+      <c r="P598" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q598" t="n">
         <v>0.04065362455529643</v>
       </c>
-      <c r="R598" t="inlineStr"/>
+      <c r="R598" t="n">
+        <v>16.53636363636364</v>
+      </c>
       <c r="S598" t="n">
         <v>1.777777777777778</v>
       </c>
@@ -36365,7 +36901,9 @@
       <c r="D599" t="n">
         <v>45</v>
       </c>
-      <c r="E599" t="inlineStr"/>
+      <c r="E599" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F599" t="n">
         <v>21</v>
       </c>
@@ -36535,7 +37073,9 @@
       <c r="A602" t="n">
         <v>652</v>
       </c>
-      <c r="B602" t="inlineStr"/>
+      <c r="B602" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C602" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -36577,11 +37117,15 @@
       <c r="O602" t="n">
         <v>2</v>
       </c>
-      <c r="P602" t="inlineStr"/>
+      <c r="P602" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q602" t="n">
         <v>-0.483326425268525</v>
       </c>
-      <c r="R602" t="inlineStr"/>
+      <c r="R602" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S602" t="n">
         <v>1.333333333333333</v>
       </c>
@@ -36771,7 +37315,9 @@
       <c r="A606" t="n">
         <v>656</v>
       </c>
-      <c r="B606" t="inlineStr"/>
+      <c r="B606" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C606" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -36813,11 +37359,15 @@
       <c r="O606" t="n">
         <v>3</v>
       </c>
-      <c r="P606" t="inlineStr"/>
+      <c r="P606" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q606" t="n">
         <v>0.9576187117469839</v>
       </c>
-      <c r="R606" t="inlineStr"/>
+      <c r="R606" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S606" t="n">
         <v>1.416666666666667</v>
       </c>
@@ -36963,7 +37513,9 @@
       <c r="F609" t="n">
         <v>32</v>
       </c>
-      <c r="G609" t="inlineStr"/>
+      <c r="G609" t="n">
+        <v>12</v>
+      </c>
       <c r="H609" t="n">
         <v>9</v>
       </c>
@@ -36997,7 +37549,9 @@
       <c r="R609" t="n">
         <v>27.625</v>
       </c>
-      <c r="S609" t="inlineStr"/>
+      <c r="S609" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="610">
       <c r="A610" t="n">
@@ -37075,7 +37629,9 @@
       <c r="D611" t="n">
         <v>40</v>
       </c>
-      <c r="E611" t="inlineStr"/>
+      <c r="E611" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F611" t="n">
         <v>22</v>
       </c>
@@ -37184,7 +37740,9 @@
       <c r="A613" t="n">
         <v>663</v>
       </c>
-      <c r="B613" t="inlineStr"/>
+      <c r="B613" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C613" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -37226,11 +37784,15 @@
       <c r="O613" t="n">
         <v>14</v>
       </c>
-      <c r="P613" t="inlineStr"/>
+      <c r="P613" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q613" t="n">
         <v>0.4336386619231625</v>
       </c>
-      <c r="R613" t="inlineStr"/>
+      <c r="R613" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S613" t="n">
         <v>0.75</v>
       </c>
@@ -37422,7 +37984,9 @@
       <c r="A617" t="n">
         <v>667</v>
       </c>
-      <c r="B617" t="inlineStr"/>
+      <c r="B617" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C617" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -37464,11 +38028,15 @@
       <c r="O617" t="n">
         <v>4</v>
       </c>
-      <c r="P617" t="inlineStr"/>
+      <c r="P617" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q617" t="n">
         <v>0.3026436494672071</v>
       </c>
-      <c r="R617" t="inlineStr"/>
+      <c r="R617" t="n">
+        <v>21.15116279069768</v>
+      </c>
       <c r="S617" t="n">
         <v>1.777777777777778</v>
       </c>
@@ -37549,7 +38117,9 @@
       <c r="D619" t="n">
         <v>60</v>
       </c>
-      <c r="E619" t="inlineStr"/>
+      <c r="E619" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F619" t="n">
         <v>40</v>
       </c>
@@ -37597,7 +38167,9 @@
       <c r="A620" t="n">
         <v>670</v>
       </c>
-      <c r="B620" t="inlineStr"/>
+      <c r="B620" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C620" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -37639,11 +38211,15 @@
       <c r="O620" t="n">
         <v>1</v>
       </c>
-      <c r="P620" t="inlineStr"/>
+      <c r="P620" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q620" t="n">
         <v>-0.09034138790065893</v>
       </c>
-      <c r="R620" t="inlineStr"/>
+      <c r="R620" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S620" t="n">
         <v>0.7368421052631579</v>
       </c>
@@ -37846,7 +38422,9 @@
       <c r="D624" t="n">
         <v>40</v>
       </c>
-      <c r="E624" t="inlineStr"/>
+      <c r="E624" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F624" t="n">
         <v>32</v>
       </c>
@@ -37966,7 +38544,9 @@
       <c r="D626" t="n">
         <v>50</v>
       </c>
-      <c r="E626" t="inlineStr"/>
+      <c r="E626" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F626" t="n">
         <v>41</v>
       </c>
@@ -38532,7 +39112,9 @@
       <c r="K635" t="n">
         <v>1</v>
       </c>
-      <c r="L635" t="inlineStr"/>
+      <c r="L635" t="n">
+        <v>0</v>
+      </c>
       <c r="M635" t="n">
         <v>0</v>
       </c>
@@ -38774,7 +39356,9 @@
       <c r="K639" t="n">
         <v>1</v>
       </c>
-      <c r="L639" t="inlineStr"/>
+      <c r="L639" t="n">
+        <v>0</v>
+      </c>
       <c r="M639" t="n">
         <v>1</v>
       </c>
@@ -38955,7 +39539,9 @@
       <c r="K642" t="n">
         <v>1</v>
       </c>
-      <c r="L642" t="inlineStr"/>
+      <c r="L642" t="n">
+        <v>0</v>
+      </c>
       <c r="M642" t="n">
         <v>0</v>
       </c>
@@ -39023,7 +39609,9 @@
       <c r="N643" t="n">
         <v>1</v>
       </c>
-      <c r="O643" t="inlineStr"/>
+      <c r="O643" t="n">
+        <v>2</v>
+      </c>
       <c r="P643" t="n">
         <v>0.4538392590379444</v>
       </c>
@@ -39041,7 +39629,9 @@
       <c r="A644" t="n">
         <v>697</v>
       </c>
-      <c r="B644" t="inlineStr"/>
+      <c r="B644" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C644" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -39083,11 +39673,15 @@
       <c r="O644" t="n">
         <v>6</v>
       </c>
-      <c r="P644" t="inlineStr"/>
+      <c r="P644" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q644" t="n">
         <v>-0.09034138790065893</v>
       </c>
-      <c r="R644" t="inlineStr"/>
+      <c r="R644" t="n">
+        <v>17.49038461538462</v>
+      </c>
       <c r="S644" t="n">
         <v>0.6470588235294118</v>
       </c>
@@ -39218,7 +39812,9 @@
       <c r="A647" t="n">
         <v>701</v>
       </c>
-      <c r="B647" t="inlineStr"/>
+      <c r="B647" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C647" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -39260,11 +39856,15 @@
       <c r="O647" t="n">
         <v>3</v>
       </c>
-      <c r="P647" t="inlineStr"/>
+      <c r="P647" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q647" t="n">
         <v>-0.2213364003566143</v>
       </c>
-      <c r="R647" t="inlineStr"/>
+      <c r="R647" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S647" t="n">
         <v>0.6666666666666666</v>
       </c>
@@ -39305,7 +39905,9 @@
       <c r="K648" t="n">
         <v>0</v>
       </c>
-      <c r="L648" t="inlineStr"/>
+      <c r="L648" t="n">
+        <v>0</v>
+      </c>
       <c r="M648" t="n">
         <v>0</v>
       </c>
@@ -39352,7 +39954,9 @@
       <c r="G649" t="n">
         <v>12</v>
       </c>
-      <c r="H649" t="inlineStr"/>
+      <c r="H649" t="n">
+        <v>11</v>
+      </c>
       <c r="I649" t="n">
         <v>8</v>
       </c>
@@ -39383,7 +39987,9 @@
       <c r="R649" t="n">
         <v>11.54</v>
       </c>
-      <c r="S649" t="inlineStr"/>
+      <c r="S649" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="650">
       <c r="A650" t="n">
@@ -39511,7 +40117,9 @@
       <c r="A652" t="n">
         <v>707</v>
       </c>
-      <c r="B652" t="inlineStr"/>
+      <c r="B652" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C652" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -39553,11 +40161,15 @@
       <c r="O652" t="n">
         <v>6</v>
       </c>
-      <c r="P652" t="inlineStr"/>
+      <c r="P652" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q652" t="n">
         <v>-0.3523314128125696</v>
       </c>
-      <c r="R652" t="inlineStr"/>
+      <c r="R652" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S652" t="n">
         <v>1</v>
       </c>
@@ -39638,7 +40250,9 @@
       <c r="D654" t="n">
         <v>34</v>
       </c>
-      <c r="E654" t="inlineStr"/>
+      <c r="E654" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F654" t="n">
         <v>22</v>
       </c>
@@ -40063,7 +40677,9 @@
       <c r="D661" t="n">
         <v>40</v>
       </c>
-      <c r="E661" t="inlineStr"/>
+      <c r="E661" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F661" t="n">
         <v>25</v>
       </c>
@@ -40326,7 +40942,9 @@
       <c r="K665" t="n">
         <v>0</v>
       </c>
-      <c r="L665" t="inlineStr"/>
+      <c r="L665" t="n">
+        <v>0</v>
+      </c>
       <c r="M665" t="n">
         <v>0</v>
       </c>
@@ -40370,7 +40988,9 @@
       <c r="F666" t="n">
         <v>49</v>
       </c>
-      <c r="G666" t="inlineStr"/>
+      <c r="G666" t="n">
+        <v>12</v>
+      </c>
       <c r="H666" t="n">
         <v>13</v>
       </c>
@@ -40404,7 +41024,9 @@
       <c r="R666" t="n">
         <v>28.875</v>
       </c>
-      <c r="S666" t="inlineStr"/>
+      <c r="S666" t="n">
+        <v>0.8571428571428571</v>
+      </c>
     </row>
     <row r="667">
       <c r="A667" t="n">
@@ -40991,7 +41613,9 @@
       <c r="K676" t="n">
         <v>1</v>
       </c>
-      <c r="L676" t="inlineStr"/>
+      <c r="L676" t="n">
+        <v>0</v>
+      </c>
       <c r="M676" t="n">
         <v>0</v>
       </c>
@@ -41088,7 +41712,9 @@
       <c r="D678" t="n">
         <v>35</v>
       </c>
-      <c r="E678" t="inlineStr"/>
+      <c r="E678" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F678" t="n">
         <v>45</v>
       </c>
@@ -41229,7 +41855,9 @@
       <c r="K680" t="n">
         <v>1</v>
       </c>
-      <c r="L680" t="inlineStr"/>
+      <c r="L680" t="n">
+        <v>0</v>
+      </c>
       <c r="M680" t="n">
         <v>0</v>
       </c>
@@ -41395,7 +42023,9 @@
       <c r="F683" t="n">
         <v>35</v>
       </c>
-      <c r="G683" t="inlineStr"/>
+      <c r="G683" t="n">
+        <v>12</v>
+      </c>
       <c r="H683" t="n">
         <v>9</v>
       </c>
@@ -41429,7 +42059,9 @@
       <c r="R683" t="n">
         <v>7.225</v>
       </c>
-      <c r="S683" t="inlineStr"/>
+      <c r="S683" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="684">
       <c r="A684" t="n">
@@ -41446,7 +42078,9 @@
       <c r="D684" t="n">
         <v>40</v>
       </c>
-      <c r="E684" t="inlineStr"/>
+      <c r="E684" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F684" t="n">
         <v>25</v>
       </c>
@@ -41633,7 +42267,9 @@
       <c r="F687" t="n">
         <v>18</v>
       </c>
-      <c r="G687" t="inlineStr"/>
+      <c r="G687" t="n">
+        <v>12</v>
+      </c>
       <c r="H687" t="n">
         <v>4</v>
       </c>
@@ -41667,7 +42303,9 @@
       <c r="R687" t="n">
         <v>16.25</v>
       </c>
-      <c r="S687" t="inlineStr"/>
+      <c r="S687" t="n">
+        <v>2.4</v>
+      </c>
     </row>
     <row r="688">
       <c r="A688" t="n">
@@ -41766,7 +42404,9 @@
       <c r="K689" t="n">
         <v>0</v>
       </c>
-      <c r="L689" t="inlineStr"/>
+      <c r="L689" t="n">
+        <v>0</v>
+      </c>
       <c r="M689" t="n">
         <v>0</v>
       </c>
@@ -41793,7 +42433,9 @@
       <c r="A690" t="n">
         <v>746</v>
       </c>
-      <c r="B690" t="inlineStr"/>
+      <c r="B690" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C690" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -41835,11 +42477,15 @@
       <c r="O690" t="n">
         <v>0</v>
       </c>
-      <c r="P690" t="inlineStr"/>
+      <c r="P690" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q690" t="n">
         <v>-0.2213364003566143</v>
       </c>
-      <c r="R690" t="inlineStr"/>
+      <c r="R690" t="n">
+        <v>21.65476190476191</v>
+      </c>
       <c r="S690" t="n">
         <v>1.230769230769231</v>
       </c>
@@ -42641,7 +43287,9 @@
       <c r="A704" t="n">
         <v>761</v>
       </c>
-      <c r="B704" t="inlineStr"/>
+      <c r="B704" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C704" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -42683,11 +43331,15 @@
       <c r="O704" t="n">
         <v>0</v>
       </c>
-      <c r="P704" t="inlineStr"/>
+      <c r="P704" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q704" t="n">
         <v>0.8266236992910285</v>
       </c>
-      <c r="R704" t="inlineStr"/>
+      <c r="R704" t="n">
+        <v>23.93421052631579</v>
+      </c>
       <c r="S704" t="n">
         <v>1.333333333333333</v>
       </c>
@@ -42768,7 +43420,9 @@
       <c r="D706" t="n">
         <v>50</v>
       </c>
-      <c r="E706" t="inlineStr"/>
+      <c r="E706" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F706" t="n">
         <v>38</v>
       </c>
@@ -42909,7 +43563,9 @@
       <c r="K708" t="n">
         <v>1</v>
       </c>
-      <c r="L708" t="inlineStr"/>
+      <c r="L708" t="n">
+        <v>0</v>
+      </c>
       <c r="M708" t="n">
         <v>1</v>
       </c>
@@ -43014,7 +43670,9 @@
       <c r="F710" t="n">
         <v>36</v>
       </c>
-      <c r="G710" t="inlineStr"/>
+      <c r="G710" t="n">
+        <v>12</v>
+      </c>
       <c r="H710" t="n">
         <v>9</v>
       </c>
@@ -43048,7 +43706,9 @@
       <c r="R710" t="n">
         <v>31.25</v>
       </c>
-      <c r="S710" t="inlineStr"/>
+      <c r="S710" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="711">
       <c r="A711" t="n">
@@ -43248,7 +43908,9 @@
       <c r="D714" t="n">
         <v>40</v>
       </c>
-      <c r="E714" t="inlineStr"/>
+      <c r="E714" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F714" t="n">
         <v>20</v>
       </c>
@@ -43357,7 +44019,9 @@
       <c r="A716" t="n">
         <v>773</v>
       </c>
-      <c r="B716" t="inlineStr"/>
+      <c r="B716" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C716" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -43399,11 +44063,15 @@
       <c r="O716" t="n">
         <v>2</v>
       </c>
-      <c r="P716" t="inlineStr"/>
+      <c r="P716" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q716" t="n">
         <v>0.8266236992910285</v>
       </c>
-      <c r="R716" t="inlineStr"/>
+      <c r="R716" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S716" t="n">
         <v>1.25</v>
       </c>
@@ -44271,7 +44939,9 @@
       <c r="D731" t="n">
         <v>40</v>
       </c>
-      <c r="E731" t="inlineStr"/>
+      <c r="E731" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F731" t="n">
         <v>36</v>
       </c>
@@ -44391,7 +45061,9 @@
       <c r="D733" t="n">
         <v>40</v>
       </c>
-      <c r="E733" t="inlineStr"/>
+      <c r="E733" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F733" t="n">
         <v>44</v>
       </c>
@@ -44456,7 +45128,9 @@
       <c r="F734" t="n">
         <v>51</v>
       </c>
-      <c r="G734" t="inlineStr"/>
+      <c r="G734" t="n">
+        <v>12</v>
+      </c>
       <c r="H734" t="n">
         <v>9</v>
       </c>
@@ -44490,7 +45164,9 @@
       <c r="R734" t="n">
         <v>26.92</v>
       </c>
-      <c r="S734" t="inlineStr"/>
+      <c r="S734" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="735">
       <c r="A735" t="n">
@@ -44528,7 +45204,9 @@
       <c r="K735" t="n">
         <v>1</v>
       </c>
-      <c r="L735" t="inlineStr"/>
+      <c r="L735" t="n">
+        <v>0</v>
+      </c>
       <c r="M735" t="n">
         <v>1</v>
       </c>
@@ -44616,7 +45294,9 @@
       <c r="A737" t="n">
         <v>795</v>
       </c>
-      <c r="B737" t="inlineStr"/>
+      <c r="B737" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C737" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -44658,11 +45338,15 @@
       <c r="O737" t="n">
         <v>7</v>
       </c>
-      <c r="P737" t="inlineStr"/>
+      <c r="P737" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q737" t="n">
         <v>-2.3172565996519</v>
       </c>
-      <c r="R737" t="inlineStr"/>
+      <c r="R737" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S737" t="n">
         <v>0.7058823529411765</v>
       </c>
@@ -44825,7 +45509,9 @@
       <c r="K740" t="n">
         <v>1</v>
       </c>
-      <c r="L740" t="inlineStr"/>
+      <c r="L740" t="n">
+        <v>0</v>
+      </c>
       <c r="M740" t="n">
         <v>0</v>
       </c>
@@ -45067,7 +45753,9 @@
       <c r="K744" t="n">
         <v>1</v>
       </c>
-      <c r="L744" t="inlineStr"/>
+      <c r="L744" t="n">
+        <v>0</v>
+      </c>
       <c r="M744" t="n">
         <v>1</v>
       </c>
@@ -46634,7 +47322,9 @@
       <c r="F770" t="n">
         <v>31</v>
       </c>
-      <c r="G770" t="inlineStr"/>
+      <c r="G770" t="n">
+        <v>12</v>
+      </c>
       <c r="H770" t="n">
         <v>17</v>
       </c>
@@ -46668,7 +47358,9 @@
       <c r="R770" t="n">
         <v>14.375</v>
       </c>
-      <c r="S770" t="inlineStr"/>
+      <c r="S770" t="n">
+        <v>0.6666666666666666</v>
+      </c>
     </row>
     <row r="771">
       <c r="A771" t="n">
@@ -46694,7 +47386,9 @@
       <c r="G771" t="n">
         <v>16</v>
       </c>
-      <c r="H771" t="inlineStr"/>
+      <c r="H771" t="n">
+        <v>11</v>
+      </c>
       <c r="I771" t="n">
         <v>2</v>
       </c>
@@ -46725,7 +47419,9 @@
       <c r="R771" t="n">
         <v>20.4</v>
       </c>
-      <c r="S771" t="inlineStr"/>
+      <c r="S771" t="n">
+        <v>1.333333333333333</v>
+      </c>
     </row>
     <row r="772">
       <c r="A772" t="n">
@@ -46824,7 +47520,9 @@
       <c r="K773" t="n">
         <v>1</v>
       </c>
-      <c r="L773" t="inlineStr"/>
+      <c r="L773" t="n">
+        <v>0</v>
+      </c>
       <c r="M773" t="n">
         <v>1</v>
       </c>
@@ -46944,7 +47642,9 @@
       <c r="K775" t="n">
         <v>1</v>
       </c>
-      <c r="L775" t="inlineStr"/>
+      <c r="L775" t="n">
+        <v>0</v>
+      </c>
       <c r="M775" t="n">
         <v>0</v>
       </c>
@@ -46971,7 +47671,9 @@
       <c r="A776" t="n">
         <v>836</v>
       </c>
-      <c r="B776" t="inlineStr"/>
+      <c r="B776" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C776" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -47013,11 +47715,15 @@
       <c r="O776" t="n">
         <v>2</v>
       </c>
-      <c r="P776" t="inlineStr"/>
+      <c r="P776" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q776" t="n">
         <v>0.4336386619231625</v>
       </c>
-      <c r="R776" t="inlineStr"/>
+      <c r="R776" t="n">
+        <v>20.21111111111111</v>
+      </c>
       <c r="S776" t="n">
         <v>2.25</v>
       </c>
@@ -47087,7 +47793,9 @@
       <c r="A778" t="n">
         <v>838</v>
       </c>
-      <c r="B778" t="inlineStr"/>
+      <c r="B778" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C778" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -47129,11 +47837,15 @@
       <c r="O778" t="n">
         <v>0</v>
       </c>
-      <c r="P778" t="inlineStr"/>
+      <c r="P778" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q778" t="n">
         <v>-0.2213364003566143</v>
       </c>
-      <c r="R778" t="inlineStr"/>
+      <c r="R778" t="n">
+        <v>30.31666666666667</v>
+      </c>
       <c r="S778" t="n">
         <v>1.888888888888889</v>
       </c>
@@ -47586,7 +48298,9 @@
       <c r="F786" t="n">
         <v>26</v>
       </c>
-      <c r="G786" t="inlineStr"/>
+      <c r="G786" t="n">
+        <v>12</v>
+      </c>
       <c r="H786" t="n">
         <v>9</v>
       </c>
@@ -47620,7 +48334,9 @@
       <c r="R786" t="n">
         <v>18.34285714285714</v>
       </c>
-      <c r="S786" t="inlineStr"/>
+      <c r="S786" t="n">
+        <v>1.2</v>
+      </c>
     </row>
     <row r="787">
       <c r="A787" t="n">
@@ -48092,7 +48808,9 @@
       <c r="N794" t="n">
         <v>1</v>
       </c>
-      <c r="O794" t="inlineStr"/>
+      <c r="O794" t="n">
+        <v>2</v>
+      </c>
       <c r="P794" t="n">
         <v>0.1843441888258141</v>
       </c>
@@ -48142,7 +48860,9 @@
       <c r="K795" t="n">
         <v>1</v>
       </c>
-      <c r="L795" t="inlineStr"/>
+      <c r="L795" t="n">
+        <v>0</v>
+      </c>
       <c r="M795" t="n">
         <v>1</v>
       </c>
@@ -48352,7 +49072,9 @@
       <c r="A799" t="n">
         <v>861</v>
       </c>
-      <c r="B799" t="inlineStr"/>
+      <c r="B799" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C799" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -48394,11 +49116,15 @@
       <c r="O799" t="n">
         <v>1</v>
       </c>
-      <c r="P799" t="inlineStr"/>
+      <c r="P799" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q799" t="n">
         <v>-0.7453164501804357</v>
       </c>
-      <c r="R799" t="inlineStr"/>
+      <c r="R799" t="n">
+        <v>18.19</v>
+      </c>
       <c r="S799" t="n">
         <v>2.6</v>
       </c>
@@ -48424,7 +49150,9 @@
       <c r="F800" t="n">
         <v>33</v>
       </c>
-      <c r="G800" t="inlineStr"/>
+      <c r="G800" t="n">
+        <v>12</v>
+      </c>
       <c r="H800" t="n">
         <v>12</v>
       </c>
@@ -48458,7 +49186,9 @@
       <c r="R800" t="n">
         <v>41.48571428571429</v>
       </c>
-      <c r="S800" t="inlineStr"/>
+      <c r="S800" t="n">
+        <v>0.9230769230769231</v>
+      </c>
     </row>
     <row r="801">
       <c r="A801" t="n">
@@ -49072,7 +49802,9 @@
       <c r="A811" t="n">
         <v>873</v>
       </c>
-      <c r="B811" t="inlineStr"/>
+      <c r="B811" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C811" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -49114,11 +49846,15 @@
       <c r="O811" t="n">
         <v>0</v>
       </c>
-      <c r="P811" t="inlineStr"/>
+      <c r="P811" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q811" t="n">
         <v>-0.483326425268525</v>
       </c>
-      <c r="R811" t="inlineStr"/>
+      <c r="R811" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S811" t="n">
         <v>0.8571428571428571</v>
       </c>
@@ -49717,7 +50453,9 @@
       <c r="N821" t="n">
         <v>1</v>
       </c>
-      <c r="O821" t="inlineStr"/>
+      <c r="O821" t="n">
+        <v>2</v>
+      </c>
       <c r="P821" t="n">
         <v>0.2046608903495667</v>
       </c>
@@ -49874,7 +50612,9 @@
       <c r="F824" t="n">
         <v>24</v>
       </c>
-      <c r="G824" t="inlineStr"/>
+      <c r="G824" t="n">
+        <v>12</v>
+      </c>
       <c r="H824" t="n">
         <v>12</v>
       </c>
@@ -49908,7 +50648,9 @@
       <c r="R824" t="n">
         <v>11.60526315789474</v>
       </c>
-      <c r="S824" t="inlineStr"/>
+      <c r="S824" t="n">
+        <v>0.9230769230769231</v>
+      </c>
     </row>
     <row r="825">
       <c r="A825" t="n">
@@ -50158,7 +50900,9 @@
       <c r="A829" t="n">
         <v>891</v>
       </c>
-      <c r="B829" t="inlineStr"/>
+      <c r="B829" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C829" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -50200,11 +50944,15 @@
       <c r="O829" t="n">
         <v>3</v>
       </c>
-      <c r="P829" t="inlineStr"/>
+      <c r="P829" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q829" t="n">
         <v>0.5646336743791178</v>
       </c>
-      <c r="R829" t="inlineStr"/>
+      <c r="R829" t="n">
+        <v>18.19</v>
+      </c>
       <c r="S829" t="n">
         <v>1.5</v>
       </c>
@@ -50213,7 +50961,9 @@
       <c r="A830" t="n">
         <v>892</v>
       </c>
-      <c r="B830" t="inlineStr"/>
+      <c r="B830" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C830" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -50255,11 +51005,15 @@
       <c r="O830" t="n">
         <v>4</v>
       </c>
-      <c r="P830" t="inlineStr"/>
+      <c r="P830" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q830" t="n">
         <v>0.5646336743791178</v>
       </c>
-      <c r="R830" t="inlineStr"/>
+      <c r="R830" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S830" t="n">
         <v>0.6666666666666666</v>
       </c>
@@ -50767,7 +51521,9 @@
       <c r="D839" t="n">
         <v>40</v>
       </c>
-      <c r="E839" t="inlineStr"/>
+      <c r="E839" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F839" t="n">
         <v>15</v>
       </c>
@@ -50896,7 +51652,9 @@
       <c r="G841" t="n">
         <v>11</v>
       </c>
-      <c r="H841" t="inlineStr"/>
+      <c r="H841" t="n">
+        <v>11</v>
+      </c>
       <c r="I841" t="n">
         <v>3</v>
       </c>
@@ -50927,7 +51685,9 @@
       <c r="R841" t="n">
         <v>10</v>
       </c>
-      <c r="S841" t="inlineStr"/>
+      <c r="S841" t="n">
+        <v>0.9166666666666666</v>
+      </c>
     </row>
     <row r="842">
       <c r="A842" t="n">
@@ -51268,7 +52028,9 @@
       <c r="K847" t="n">
         <v>0</v>
       </c>
-      <c r="L847" t="inlineStr"/>
+      <c r="L847" t="n">
+        <v>0</v>
+      </c>
       <c r="M847" t="n">
         <v>0</v>
       </c>
@@ -51356,7 +52118,9 @@
       <c r="A849" t="n">
         <v>912</v>
       </c>
-      <c r="B849" t="inlineStr"/>
+      <c r="B849" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C849" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -51398,11 +52162,15 @@
       <c r="O849" t="n">
         <v>1</v>
       </c>
-      <c r="P849" t="inlineStr"/>
+      <c r="P849" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q849" t="n">
         <v>0.1716486370112518</v>
       </c>
-      <c r="R849" t="inlineStr"/>
+      <c r="R849" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S849" t="n">
         <v>1.3</v>
       </c>
@@ -51411,7 +52179,9 @@
       <c r="A850" t="n">
         <v>913</v>
       </c>
-      <c r="B850" t="inlineStr"/>
+      <c r="B850" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C850" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -51453,11 +52223,15 @@
       <c r="O850" t="n">
         <v>1</v>
       </c>
-      <c r="P850" t="inlineStr"/>
+      <c r="P850" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q850" t="n">
         <v>0.3026436494672071</v>
       </c>
-      <c r="R850" t="inlineStr"/>
+      <c r="R850" t="n">
+        <v>20.21111111111111</v>
+      </c>
       <c r="S850" t="n">
         <v>1.285714285714286</v>
       </c>
@@ -51538,7 +52312,9 @@
       <c r="D852" t="n">
         <v>45</v>
       </c>
-      <c r="E852" t="inlineStr"/>
+      <c r="E852" t="n">
+        <v>101.2327790973872</v>
+      </c>
       <c r="F852" t="n">
         <v>40</v>
       </c>
@@ -51586,7 +52362,9 @@
       <c r="A853" t="n">
         <v>916</v>
       </c>
-      <c r="B853" t="inlineStr"/>
+      <c r="B853" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C853" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -51628,11 +52406,15 @@
       <c r="O853" t="n">
         <v>0</v>
       </c>
-      <c r="P853" t="inlineStr"/>
+      <c r="P853" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q853" t="n">
         <v>0.8266236992910285</v>
       </c>
-      <c r="R853" t="inlineStr"/>
+      <c r="R853" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S853" t="n">
         <v>1.230769230769231</v>
       </c>
@@ -51641,7 +52423,9 @@
       <c r="A854" t="n">
         <v>918</v>
       </c>
-      <c r="B854" t="inlineStr"/>
+      <c r="B854" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C854" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -51683,11 +52467,15 @@
       <c r="O854" t="n">
         <v>3</v>
       </c>
-      <c r="P854" t="inlineStr"/>
+      <c r="P854" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q854" t="n">
         <v>-0.876311462636391</v>
       </c>
-      <c r="R854" t="inlineStr"/>
+      <c r="R854" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S854" t="n">
         <v>2.666666666666667</v>
       </c>
@@ -52079,7 +52867,9 @@
       <c r="F861" t="n">
         <v>37</v>
       </c>
-      <c r="G861" t="inlineStr"/>
+      <c r="G861" t="n">
+        <v>12</v>
+      </c>
       <c r="H861" t="n">
         <v>13</v>
       </c>
@@ -52113,7 +52903,9 @@
       <c r="R861" t="n">
         <v>25.64444444444445</v>
       </c>
-      <c r="S861" t="inlineStr"/>
+      <c r="S861" t="n">
+        <v>0.8571428571428571</v>
+      </c>
     </row>
     <row r="862">
       <c r="A862" t="n">
@@ -52136,7 +52928,9 @@
       <c r="F862" t="n">
         <v>47</v>
       </c>
-      <c r="G862" t="inlineStr"/>
+      <c r="G862" t="n">
+        <v>12</v>
+      </c>
       <c r="H862" t="n">
         <v>18</v>
       </c>
@@ -52170,13 +52964,17 @@
       <c r="R862" t="n">
         <v>24.68888888888889</v>
       </c>
-      <c r="S862" t="inlineStr"/>
+      <c r="S862" t="n">
+        <v>0.631578947368421</v>
+      </c>
     </row>
     <row r="863">
       <c r="A863" t="n">
         <v>927</v>
       </c>
-      <c r="B863" t="inlineStr"/>
+      <c r="B863" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C863" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -52218,11 +53016,15 @@
       <c r="O863" t="n">
         <v>6</v>
       </c>
-      <c r="P863" t="inlineStr"/>
+      <c r="P863" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q863" t="n">
         <v>0.04065362455529643</v>
       </c>
-      <c r="R863" t="inlineStr"/>
+      <c r="R863" t="n">
+        <v>23.93421052631579</v>
+      </c>
       <c r="S863" t="n">
         <v>0.8571428571428571</v>
       </c>
@@ -52471,7 +53273,9 @@
       <c r="A868" t="n">
         <v>932</v>
       </c>
-      <c r="B868" t="inlineStr"/>
+      <c r="B868" t="n">
+        <v>909.5</v>
+      </c>
       <c r="C868" t="inlineStr">
         <is>
           <t>BAJO</t>
@@ -52513,11 +53317,15 @@
       <c r="O868" t="n">
         <v>1</v>
       </c>
-      <c r="P868" t="inlineStr"/>
+      <c r="P868" t="n">
+        <v>0.2373767553032566</v>
+      </c>
       <c r="Q868" t="n">
         <v>-0.483326425268525</v>
       </c>
-      <c r="R868" t="inlineStr"/>
+      <c r="R868" t="n">
+        <v>22.7375</v>
+      </c>
       <c r="S868" t="n">
         <v>1.4</v>
       </c>

</xml_diff>